<commit_message>
Reporte muestra TODAS las actividades por defecto, fechas para filtrar
</commit_message>
<xml_diff>
--- a/ASISTENCIA/puntualidad.xlsx
+++ b/ASISTENCIA/puntualidad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose Alonso\IntelliJ_IDEA\work_manage_app\ASISTENCIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF7259F3-1DAF-4FD0-9288-ACE5009EACF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8812B9D9-BB55-443B-A941-3EFC33CC48DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8BB8B4E3-A626-477D-80D2-DB6757049F7D}"/>
   </bookViews>
@@ -34,6 +34,107 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+  <si>
+    <t>CAPATAZ</t>
+  </si>
+  <si>
+    <t>OPERARIO</t>
+  </si>
+  <si>
+    <t>OFICIAL</t>
+  </si>
+  <si>
+    <t>PEON</t>
+  </si>
+  <si>
+    <t>GUARDIAN</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>PERSONAL</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -84,6 +185,42 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E5A757A7-F768-42AB-BB4B-A81FB06274BF}" name="Tabla3" displayName="Tabla3" ref="A1:AA6" totalsRowShown="0">
+  <autoFilter ref="A1:AA6" xr:uid="{E5A757A7-F768-42AB-BB4B-A81FB06274BF}"/>
+  <tableColumns count="27">
+    <tableColumn id="1" xr3:uid="{008E7CDC-1181-4772-A7BC-26796E8B7E26}" name="PERSONAL"/>
+    <tableColumn id="2" xr3:uid="{88B0D090-0409-40F1-B3AB-A92D4C3635D1}" name="3"/>
+    <tableColumn id="3" xr3:uid="{285A39AC-732C-435D-8F3A-503A79858FCB}" name="4"/>
+    <tableColumn id="4" xr3:uid="{B1ACDE91-CE85-44B6-AAD2-09AC0C9779C4}" name="5"/>
+    <tableColumn id="5" xr3:uid="{72E7A36E-3DA6-4A03-9A53-49D6CD7AF6C2}" name="6"/>
+    <tableColumn id="6" xr3:uid="{0BB81B4A-B517-4518-90E1-9710C5E63903}" name="7"/>
+    <tableColumn id="7" xr3:uid="{A130B706-2B7E-4990-843E-CF6DE9735002}" name="8"/>
+    <tableColumn id="8" xr3:uid="{E50DA4E5-0FCB-4F49-9E4F-CFF5C5B48D8B}" name="9"/>
+    <tableColumn id="9" xr3:uid="{AE1DB262-36D4-4C6D-94FE-27EB6815DCAA}" name="10"/>
+    <tableColumn id="10" xr3:uid="{4FCBB51E-2828-4EDB-A05C-84FDC6A7AB92}" name="11"/>
+    <tableColumn id="11" xr3:uid="{C928FE5F-7477-44E4-A76B-25DAC1CFAE6C}" name="12"/>
+    <tableColumn id="12" xr3:uid="{F9869971-8073-412D-B82F-31DF00D2BF66}" name="13"/>
+    <tableColumn id="13" xr3:uid="{0A6BBD4F-D710-438D-9226-83703D76677D}" name="14"/>
+    <tableColumn id="14" xr3:uid="{341B34B8-4846-48DC-8537-E2F17D937214}" name="15"/>
+    <tableColumn id="15" xr3:uid="{60351B35-F6A6-4D0E-A0C4-A90BB53BC849}" name="16"/>
+    <tableColumn id="16" xr3:uid="{5BC57F69-D843-4D15-8CE1-CB48FBB9E1C0}" name="17"/>
+    <tableColumn id="17" xr3:uid="{DFC4A4F4-0F34-4AD3-8CC4-D7C1FB29C685}" name="18"/>
+    <tableColumn id="18" xr3:uid="{0D275F14-8510-409F-A731-076470B7372A}" name="19"/>
+    <tableColumn id="19" xr3:uid="{1FAED0BA-BF23-4DFE-8756-BBCA4719A044}" name="20"/>
+    <tableColumn id="20" xr3:uid="{F34B898D-A5DD-40BF-B81E-0F2E45DAA1A4}" name="21"/>
+    <tableColumn id="21" xr3:uid="{FB377D86-DFBF-4022-AB72-DF5078BFA66A}" name="22"/>
+    <tableColumn id="22" xr3:uid="{F90991D2-D210-4FD1-9DA1-C389C63BD828}" name="23"/>
+    <tableColumn id="23" xr3:uid="{83F1659A-31CA-4A38-94B7-A970CE333139}" name="24"/>
+    <tableColumn id="24" xr3:uid="{A4B19233-2527-4EF9-8D63-92530FE31B6C}" name="25"/>
+    <tableColumn id="25" xr3:uid="{0DDB12C8-2CFD-4F83-8F74-C7629D265E8B}" name="26"/>
+    <tableColumn id="26" xr3:uid="{A2B90219-630A-46D9-B93A-1999292C165E}" name="27"/>
+    <tableColumn id="27" xr3:uid="{7C7BFE46-9376-48D5-BCDA-FA76EAC7CE52}" name="28"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -383,9 +520,515 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D622D51-97E8-436E-8008-2A57C83E6D78}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="8" width="4.77734375" customWidth="1"/>
+    <col min="9" max="27" width="4.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" t="s">
+        <v>18</v>
+      </c>
+      <c r="P1" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>20</v>
+      </c>
+      <c r="R1" t="s">
+        <v>21</v>
+      </c>
+      <c r="S1" t="s">
+        <v>22</v>
+      </c>
+      <c r="T1" t="s">
+        <v>23</v>
+      </c>
+      <c r="U1" t="s">
+        <v>24</v>
+      </c>
+      <c r="V1" t="s">
+        <v>25</v>
+      </c>
+      <c r="W1" t="s">
+        <v>26</v>
+      </c>
+      <c r="X1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>1</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>1</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
+      </c>
+      <c r="T2">
+        <v>1</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>1</v>
+      </c>
+      <c r="X2">
+        <v>1</v>
+      </c>
+      <c r="Y2">
+        <v>1</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>11</v>
+      </c>
+      <c r="C3">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>14</v>
+      </c>
+      <c r="E3">
+        <v>14</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>15</v>
+      </c>
+      <c r="I3">
+        <v>15</v>
+      </c>
+      <c r="J3">
+        <v>15</v>
+      </c>
+      <c r="K3">
+        <v>15</v>
+      </c>
+      <c r="L3">
+        <v>15</v>
+      </c>
+      <c r="M3">
+        <v>15</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>14</v>
+      </c>
+      <c r="P3">
+        <v>15</v>
+      </c>
+      <c r="Q3">
+        <v>15</v>
+      </c>
+      <c r="R3">
+        <v>15</v>
+      </c>
+      <c r="S3">
+        <v>15</v>
+      </c>
+      <c r="T3">
+        <v>15</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>15</v>
+      </c>
+      <c r="W3">
+        <v>15</v>
+      </c>
+      <c r="X3">
+        <v>14</v>
+      </c>
+      <c r="Y3">
+        <v>15</v>
+      </c>
+      <c r="Z3">
+        <v>13</v>
+      </c>
+      <c r="AA3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>9</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>10</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>11</v>
+      </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
+      <c r="J4">
+        <v>12</v>
+      </c>
+      <c r="K4">
+        <v>12</v>
+      </c>
+      <c r="L4">
+        <v>12</v>
+      </c>
+      <c r="M4">
+        <v>12</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>12</v>
+      </c>
+      <c r="P4">
+        <v>13</v>
+      </c>
+      <c r="Q4">
+        <v>13</v>
+      </c>
+      <c r="R4">
+        <v>13</v>
+      </c>
+      <c r="S4">
+        <v>13</v>
+      </c>
+      <c r="T4">
+        <v>13</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>13</v>
+      </c>
+      <c r="W4">
+        <v>13</v>
+      </c>
+      <c r="X4">
+        <v>12</v>
+      </c>
+      <c r="Y4">
+        <v>13</v>
+      </c>
+      <c r="Z4">
+        <v>13</v>
+      </c>
+      <c r="AA4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>9</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>9</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>9</v>
+      </c>
+      <c r="I5">
+        <v>9</v>
+      </c>
+      <c r="J5">
+        <v>9</v>
+      </c>
+      <c r="K5">
+        <v>9</v>
+      </c>
+      <c r="L5">
+        <v>9</v>
+      </c>
+      <c r="M5">
+        <v>8</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>7</v>
+      </c>
+      <c r="P5">
+        <v>8</v>
+      </c>
+      <c r="Q5">
+        <v>8</v>
+      </c>
+      <c r="R5">
+        <v>8</v>
+      </c>
+      <c r="S5">
+        <v>8</v>
+      </c>
+      <c r="T5">
+        <v>8</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>7</v>
+      </c>
+      <c r="W5">
+        <v>8</v>
+      </c>
+      <c r="X5">
+        <v>8</v>
+      </c>
+      <c r="Y5">
+        <v>8</v>
+      </c>
+      <c r="Z5">
+        <v>8</v>
+      </c>
+      <c r="AA5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>3</v>
+      </c>
+      <c r="P6">
+        <v>3</v>
+      </c>
+      <c r="Q6">
+        <v>3</v>
+      </c>
+      <c r="R6">
+        <v>3</v>
+      </c>
+      <c r="S6">
+        <v>3</v>
+      </c>
+      <c r="T6">
+        <v>3</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>3</v>
+      </c>
+      <c r="W6">
+        <v>3</v>
+      </c>
+      <c r="X6">
+        <v>3</v>
+      </c>
+      <c r="Y6">
+        <v>3</v>
+      </c>
+      <c r="Z6">
+        <v>3</v>
+      </c>
+      <c r="AA6">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>